<commit_message>
Add CARGO classification (DURIAN vs NON DURIAN) to TOTAL RH and Dashboard
New stat-card section on TOTAL RH, below the Year x Brand x Size
matrix: DURIAN = 40'RH built 2021-2026, NON DURIAN = built <=2020,
both depots combined, live SUMs over the matrix. Dashboard gets two
matching KPI cards that link to these cells rather than recomputing.

Moved the stat_card/draw_card_border helpers up so both sheets can
share them instead of duplicating the Dashboard-only copies.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_9-22.xlsx
+++ b/Stock_Daily_Reefer_9-22.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,22 +49,32 @@
     <font/>
     <font>
       <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008B979C"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="00C62828"/>
       <sz val="20"/>
-    </font>
-    <font>
-      <color rgb="00808080"/>
-      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -156,6 +166,23 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008B979C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00C62828"/>
       <sz val="11"/>
     </font>
@@ -163,11 +190,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001A1A1A"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00808080"/>
       <sz val="11"/>
     </font>
     <font>
@@ -412,134 +434,153 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4062,7 +4103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4088,16 +4129,16 @@
         <f>"Stock vs Booking Report - Reefer (20'RE / 40'RH)  as of "&amp;DAY(Control!$B$1)&amp;" "&amp;CHOOSE(MONTH(Control!$B$1),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;" "&amp;YEAR(Control!$B$1)</f>
         <v/>
       </c>
-      <c r="B1" s="51" t="n"/>
-      <c r="C1" s="51" t="n"/>
-      <c r="D1" s="51" t="n"/>
-      <c r="E1" s="51" t="n"/>
-      <c r="F1" s="51" t="n"/>
-      <c r="G1" s="51" t="n"/>
-      <c r="H1" s="51" t="n"/>
-      <c r="I1" s="51" t="n"/>
-      <c r="J1" s="51" t="n"/>
-      <c r="K1" s="52" t="n"/>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="58" t="n"/>
+      <c r="E1" s="58" t="n"/>
+      <c r="F1" s="58" t="n"/>
+      <c r="G1" s="58" t="n"/>
+      <c r="H1" s="58" t="n"/>
+      <c r="I1" s="58" t="n"/>
+      <c r="J1" s="58" t="n"/>
+      <c r="K1" s="59" t="n"/>
       <c r="L1" s="1" t="n"/>
       <c r="M1" s="1" t="n"/>
       <c r="N1" s="1" t="n"/>
@@ -4111,8 +4152,8 @@
           <t>BKK27 / BC2</t>
         </is>
       </c>
-      <c r="C2" s="51" t="n"/>
-      <c r="D2" s="52" t="n"/>
+      <c r="C2" s="58" t="n"/>
+      <c r="D2" s="59" t="n"/>
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
@@ -4121,8 +4162,8 @@
           <t>LCH27 / HAST</t>
         </is>
       </c>
-      <c r="I2" s="51" t="n"/>
-      <c r="J2" s="52" t="n"/>
+      <c r="I2" s="58" t="n"/>
+      <c r="J2" s="59" t="n"/>
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
       <c r="M2" s="5" t="inlineStr">
@@ -4394,11 +4435,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C8" s="53">
+      <c r="C8" s="60">
         <f>C4-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="54">
+      <c r="D8" s="61">
         <f>D4-D5-D6-D7</f>
         <v/>
       </c>
@@ -4409,11 +4450,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I8" s="53">
+      <c r="I8" s="60">
         <f>I4-I5-I6-I7</f>
         <v/>
       </c>
-      <c r="J8" s="53">
+      <c r="J8" s="60">
         <f>J4-J5-J6-J7</f>
         <v/>
       </c>
@@ -4492,11 +4533,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="60">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="54">
+      <c r="D10" s="61">
         <f>D8-D9</f>
         <v/>
       </c>
@@ -4507,11 +4548,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I10" s="53">
+      <c r="I10" s="60">
         <f>I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="53">
+      <c r="J10" s="60">
         <f>J8-J9</f>
         <v/>
       </c>
@@ -4580,11 +4621,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C12" s="53">
+      <c r="C12" s="60">
         <f>C10-C11</f>
         <v/>
       </c>
-      <c r="D12" s="54">
+      <c r="D12" s="61">
         <f>D10-D11</f>
         <v/>
       </c>
@@ -4595,11 +4636,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I12" s="53">
+      <c r="I12" s="60">
         <f>I10-I11</f>
         <v/>
       </c>
-      <c r="J12" s="54">
+      <c r="J12" s="61">
         <f>J10-J11</f>
         <v/>
       </c>
@@ -4849,9 +4890,9 @@
           <t>BKK / BC2 (BKK27)</t>
         </is>
       </c>
-      <c r="C20" s="51" t="n"/>
-      <c r="D20" s="51" t="n"/>
-      <c r="E20" s="52" t="n"/>
+      <c r="C20" s="58" t="n"/>
+      <c r="D20" s="58" t="n"/>
+      <c r="E20" s="59" t="n"/>
       <c r="F20" s="1" t="n"/>
       <c r="G20" s="1" t="n"/>
       <c r="H20" s="17" t="inlineStr">
@@ -4859,9 +4900,9 @@
           <t>LCH / HAST (LCH27)</t>
         </is>
       </c>
-      <c r="I20" s="51" t="n"/>
-      <c r="J20" s="51" t="n"/>
-      <c r="K20" s="52" t="n"/>
+      <c r="I20" s="58" t="n"/>
+      <c r="J20" s="58" t="n"/>
+      <c r="K20" s="59" t="n"/>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="n"/>
@@ -4922,7 +4963,7 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="55" t="n"/>
+      <c r="B22" s="62" t="n"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -4940,7 +4981,7 @@
       </c>
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
-      <c r="H22" s="55" t="n"/>
+      <c r="H22" s="62" t="n"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -5277,24 +5318,24 @@
           <t>BKK27 / BC2  —  Stock by Built Year x Brand x Size</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n"/>
-      <c r="D33" s="51" t="n"/>
-      <c r="E33" s="51" t="n"/>
-      <c r="F33" s="51" t="n"/>
-      <c r="G33" s="51" t="n"/>
-      <c r="H33" s="52" t="n"/>
+      <c r="C33" s="58" t="n"/>
+      <c r="D33" s="58" t="n"/>
+      <c r="E33" s="58" t="n"/>
+      <c r="F33" s="58" t="n"/>
+      <c r="G33" s="58" t="n"/>
+      <c r="H33" s="59" t="n"/>
       <c r="I33" s="1" t="n"/>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>LCH27 / HAST  —  Stock by Built Year x Brand x Size</t>
         </is>
       </c>
-      <c r="K33" s="51" t="n"/>
-      <c r="L33" s="51" t="n"/>
-      <c r="M33" s="51" t="n"/>
-      <c r="N33" s="51" t="n"/>
-      <c r="O33" s="51" t="n"/>
-      <c r="P33" s="52" t="n"/>
+      <c r="K33" s="58" t="n"/>
+      <c r="L33" s="58" t="n"/>
+      <c r="M33" s="58" t="n"/>
+      <c r="N33" s="58" t="n"/>
+      <c r="O33" s="58" t="n"/>
+      <c r="P33" s="59" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="1" t="n"/>
@@ -5309,19 +5350,19 @@
           <t>CARRIER</t>
         </is>
       </c>
-      <c r="D34" s="52" t="n"/>
+      <c r="D34" s="59" t="n"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
-      <c r="F34" s="52" t="n"/>
+      <c r="F34" s="59" t="n"/>
       <c r="G34" s="4" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
-      <c r="H34" s="52" t="n"/>
+      <c r="H34" s="59" t="n"/>
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="18" t="inlineStr">
         <is>
@@ -5334,23 +5375,23 @@
           <t>CARRIER</t>
         </is>
       </c>
-      <c r="L34" s="52" t="n"/>
+      <c r="L34" s="59" t="n"/>
       <c r="M34" s="4" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
-      <c r="N34" s="52" t="n"/>
+      <c r="N34" s="59" t="n"/>
       <c r="O34" s="4" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
-      <c r="P34" s="52" t="n"/>
+      <c r="P34" s="59" t="n"/>
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="55" t="n"/>
+      <c r="B35" s="62" t="n"/>
       <c r="C35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
@@ -5382,7 +5423,7 @@
         </is>
       </c>
       <c r="I35" s="1" t="n"/>
-      <c r="J35" s="55" t="n"/>
+      <c r="J35" s="62" t="n"/>
       <c r="K35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
@@ -5899,6 +5940,140 @@
       </c>
       <c r="O53" s="13" t="n"/>
       <c r="P53" s="13" t="n"/>
+    </row>
+    <row r="54" ht="13" customHeight="1">
+      <c r="A54" s="1" t="n"/>
+      <c r="B54" s="1" t="n"/>
+      <c r="C54" s="1" t="n"/>
+      <c r="D54" s="1" t="n"/>
+      <c r="E54" s="1" t="n"/>
+      <c r="F54" s="1" t="n"/>
+      <c r="G54" s="1" t="n"/>
+      <c r="H54" s="1" t="n"/>
+      <c r="I54" s="1" t="n"/>
+      <c r="J54" s="1" t="n"/>
+      <c r="K54" s="1" t="n"/>
+      <c r="L54" s="1" t="n"/>
+      <c r="M54" s="1" t="n"/>
+      <c r="N54" s="1" t="n"/>
+      <c r="O54" s="1" t="n"/>
+      <c r="P54" s="1" t="n"/>
+    </row>
+    <row r="55" ht="13" customHeight="1">
+      <c r="A55" s="1" t="n"/>
+      <c r="B55" s="1" t="n"/>
+      <c r="C55" s="1" t="n"/>
+      <c r="D55" s="1" t="n"/>
+      <c r="E55" s="1" t="n"/>
+      <c r="F55" s="1" t="n"/>
+      <c r="G55" s="1" t="n"/>
+      <c r="H55" s="1" t="n"/>
+      <c r="I55" s="1" t="n"/>
+      <c r="J55" s="1" t="n"/>
+      <c r="K55" s="1" t="n"/>
+      <c r="L55" s="1" t="n"/>
+      <c r="M55" s="1" t="n"/>
+      <c r="N55" s="1" t="n"/>
+      <c r="O55" s="1" t="n"/>
+      <c r="P55" s="1" t="n"/>
+    </row>
+    <row r="56" ht="13" customHeight="1">
+      <c r="A56" s="1" t="n"/>
+      <c r="B56" s="31" t="inlineStr">
+        <is>
+          <t>CARGO CLASSIFICATION  (both depots, 40'RH stock, by Built Year)</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="n"/>
+      <c r="D56" s="1" t="n"/>
+      <c r="E56" s="1" t="n"/>
+      <c r="F56" s="1" t="n"/>
+      <c r="G56" s="1" t="n"/>
+      <c r="H56" s="1" t="n"/>
+      <c r="I56" s="1" t="n"/>
+      <c r="J56" s="1" t="n"/>
+      <c r="K56" s="1" t="n"/>
+      <c r="L56" s="1" t="n"/>
+      <c r="M56" s="1" t="n"/>
+      <c r="N56" s="1" t="n"/>
+      <c r="O56" s="1" t="n"/>
+      <c r="P56" s="1" t="n"/>
+    </row>
+    <row r="57" ht="13" customHeight="1">
+      <c r="A57" s="1" t="n"/>
+      <c r="B57" s="32" t="inlineStr">
+        <is>
+          <t>DURIAN  (built 2021-2026)</t>
+        </is>
+      </c>
+      <c r="C57" s="33" t="n"/>
+      <c r="D57" s="33" t="n"/>
+      <c r="E57" s="33" t="n"/>
+      <c r="F57" s="1" t="n"/>
+      <c r="G57" s="32" t="inlineStr">
+        <is>
+          <t>NON DURIAN  (built ≤ 2020)</t>
+        </is>
+      </c>
+      <c r="H57" s="33" t="n"/>
+      <c r="I57" s="33" t="n"/>
+      <c r="J57" s="33" t="n"/>
+      <c r="K57" s="1" t="n"/>
+      <c r="L57" s="1" t="n"/>
+      <c r="M57" s="1" t="n"/>
+      <c r="N57" s="1" t="n"/>
+      <c r="O57" s="1" t="n"/>
+      <c r="P57" s="1" t="n"/>
+    </row>
+    <row r="58" ht="13" customHeight="1">
+      <c r="A58" s="1" t="n"/>
+      <c r="B58" s="34">
+        <f>SUM(D36:D41)+SUM(F36:F41)+SUM(H36:H41)+SUM(L36:L41)+SUM(N36:N41)+SUM(P36:P41)</f>
+        <v/>
+      </c>
+      <c r="C58" s="33" t="n"/>
+      <c r="D58" s="33" t="n"/>
+      <c r="E58" s="33" t="n"/>
+      <c r="F58" s="1" t="n"/>
+      <c r="G58" s="35">
+        <f>SUM(D42:D52)+SUM(F42:F52)+SUM(H42:H52)+SUM(L42:L52)+SUM(N42:N52)+SUM(P42:P52)</f>
+        <v/>
+      </c>
+      <c r="H58" s="33" t="n"/>
+      <c r="I58" s="33" t="n"/>
+      <c r="J58" s="33" t="n"/>
+      <c r="K58" s="1" t="n"/>
+      <c r="L58" s="1" t="n"/>
+      <c r="M58" s="1" t="n"/>
+      <c r="N58" s="1" t="n"/>
+      <c r="O58" s="1" t="n"/>
+      <c r="P58" s="1" t="n"/>
+    </row>
+    <row r="59" ht="13" customHeight="1">
+      <c r="A59" s="1" t="n"/>
+      <c r="B59" s="36" t="inlineStr">
+        <is>
+          <t>40'RH, both depots combined</t>
+        </is>
+      </c>
+      <c r="C59" s="33" t="n"/>
+      <c r="D59" s="33" t="n"/>
+      <c r="E59" s="33" t="n"/>
+      <c r="F59" s="1" t="n"/>
+      <c r="G59" s="36" t="inlineStr">
+        <is>
+          <t>40'RH, both depots combined</t>
+        </is>
+      </c>
+      <c r="H59" s="33" t="n"/>
+      <c r="I59" s="33" t="n"/>
+      <c r="J59" s="33" t="n"/>
+      <c r="K59" s="1" t="n"/>
+      <c r="L59" s="1" t="n"/>
+      <c r="M59" s="1" t="n"/>
+      <c r="N59" s="1" t="n"/>
+      <c r="O59" s="1" t="n"/>
+      <c r="P59" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -5930,7 +6105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P40"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5946,7 +6121,7 @@
   <sheetData>
     <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="31">
+      <c r="B1" s="37">
         <f>'TOTAL RH'!A1</f>
         <v/>
       </c>
@@ -5974,99 +6149,99 @@
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>SHORTFALL ALERT</t>
         </is>
       </c>
-      <c r="C4" s="34" t="n"/>
-      <c r="D4" s="34" t="n"/>
+      <c r="C4" s="33" t="n"/>
+      <c r="D4" s="33" t="n"/>
       <c r="E4" s="1" t="n"/>
-      <c r="F4" s="33" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>COMBINED 40'RH STOCK</t>
         </is>
       </c>
-      <c r="G4" s="34" t="n"/>
-      <c r="H4" s="34" t="n"/>
+      <c r="G4" s="33" t="n"/>
+      <c r="H4" s="33" t="n"/>
       <c r="I4" s="1" t="n"/>
-      <c r="J4" s="33" t="inlineStr">
+      <c r="J4" s="39" t="inlineStr">
         <is>
           <t>COMBINED 40'RH BOOKING</t>
         </is>
       </c>
-      <c r="K4" s="34" t="n"/>
-      <c r="L4" s="34" t="n"/>
+      <c r="K4" s="33" t="n"/>
+      <c r="L4" s="33" t="n"/>
       <c r="M4" s="1" t="n"/>
-      <c r="N4" s="33" t="inlineStr">
+      <c r="N4" s="39" t="inlineStr">
         <is>
           <t>COMBINED 40'RH BALANCE</t>
         </is>
       </c>
-      <c r="O4" s="34" t="n"/>
-      <c r="P4" s="34" t="n"/>
+      <c r="O4" s="33" t="n"/>
+      <c r="P4" s="33" t="n"/>
     </row>
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="35">
+      <c r="B5" s="40">
         <f>MIN('TOTAL RH'!D12,'TOTAL RH'!J12)</f>
         <v/>
       </c>
-      <c r="C5" s="34" t="n"/>
-      <c r="D5" s="34" t="n"/>
+      <c r="C5" s="33" t="n"/>
+      <c r="D5" s="33" t="n"/>
       <c r="E5" s="1" t="n"/>
-      <c r="F5" s="36">
+      <c r="F5" s="41">
         <f>'TOTAL RH'!O5</f>
         <v/>
       </c>
-      <c r="G5" s="34" t="n"/>
-      <c r="H5" s="34" t="n"/>
+      <c r="G5" s="33" t="n"/>
+      <c r="H5" s="33" t="n"/>
       <c r="I5" s="1" t="n"/>
-      <c r="J5" s="36">
+      <c r="J5" s="41">
         <f>'TOTAL RH'!O10</f>
         <v/>
       </c>
-      <c r="K5" s="34" t="n"/>
-      <c r="L5" s="34" t="n"/>
+      <c r="K5" s="33" t="n"/>
+      <c r="L5" s="33" t="n"/>
       <c r="M5" s="1" t="n"/>
-      <c r="N5" s="35">
+      <c r="N5" s="40">
         <f>'TOTAL RH'!O15</f>
         <v/>
       </c>
-      <c r="O5" s="34" t="n"/>
-      <c r="P5" s="34" t="n"/>
+      <c r="O5" s="33" t="n"/>
+      <c r="P5" s="33" t="n"/>
     </row>
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="37">
+      <c r="B6" s="42">
         <f>"BKK27/LCH27 40'RH, worse "&amp;'TOTAL RH'!B12</f>
         <v/>
       </c>
-      <c r="C6" s="34" t="n"/>
-      <c r="D6" s="34" t="n"/>
+      <c r="C6" s="33" t="n"/>
+      <c r="D6" s="33" t="n"/>
       <c r="E6" s="1" t="n"/>
-      <c r="F6" s="37" t="inlineStr">
+      <c r="F6" s="42" t="inlineStr">
         <is>
           <t>BKK27 + LCH27</t>
         </is>
       </c>
-      <c r="G6" s="34" t="n"/>
-      <c r="H6" s="34" t="n"/>
+      <c r="G6" s="33" t="n"/>
+      <c r="H6" s="33" t="n"/>
       <c r="I6" s="1" t="n"/>
-      <c r="J6" s="37" t="inlineStr">
+      <c r="J6" s="42" t="inlineStr">
         <is>
           <t>pending + all weeks</t>
         </is>
       </c>
-      <c r="K6" s="34" t="n"/>
-      <c r="L6" s="34" t="n"/>
+      <c r="K6" s="33" t="n"/>
+      <c r="L6" s="33" t="n"/>
       <c r="M6" s="1" t="n"/>
-      <c r="N6" s="37">
+      <c r="N6" s="42">
         <f>"pending + all weeks, both depots, "&amp;'TOTAL RH'!B12</f>
         <v/>
       </c>
-      <c r="O6" s="34" t="n"/>
-      <c r="P6" s="34" t="n"/>
+      <c r="O6" s="33" t="n"/>
+      <c r="P6" s="33" t="n"/>
     </row>
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="1" t="n"/>
@@ -6088,7 +6263,7 @@
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="38" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>DETAIL BY DEPOT</t>
         </is>
@@ -6110,21 +6285,21 @@
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="39">
+      <c r="B9" s="44">
         <f>'TOTAL RH'!B2</f>
         <v/>
       </c>
-      <c r="C9" s="56" t="n"/>
-      <c r="D9" s="57" t="n"/>
+      <c r="C9" s="63" t="n"/>
+      <c r="D9" s="64" t="n"/>
       <c r="E9" s="1" t="n"/>
       <c r="F9" s="1" t="n"/>
       <c r="G9" s="1" t="n"/>
-      <c r="H9" s="40">
+      <c r="H9" s="45">
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="I9" s="56" t="n"/>
-      <c r="J9" s="57" t="n"/>
+      <c r="I9" s="63" t="n"/>
+      <c r="J9" s="64" t="n"/>
       <c r="K9" s="1" t="n"/>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
@@ -6134,13 +6309,13 @@
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="34" t="n"/>
-      <c r="C10" s="41" t="inlineStr">
+      <c r="B10" s="33" t="n"/>
+      <c r="C10" s="46" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="46" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
@@ -6148,13 +6323,13 @@
       <c r="E10" s="1" t="n"/>
       <c r="F10" s="1" t="n"/>
       <c r="G10" s="1" t="n"/>
-      <c r="H10" s="34" t="n"/>
-      <c r="I10" s="41" t="inlineStr">
+      <c r="H10" s="33" t="n"/>
+      <c r="I10" s="46" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="J10" s="41" t="inlineStr">
+      <c r="J10" s="46" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
@@ -6168,30 +6343,30 @@
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="42">
+      <c r="B11" s="47">
         <f>'TOTAL RH'!B4</f>
         <v/>
       </c>
-      <c r="C11" s="43">
+      <c r="C11" s="48">
         <f>'TOTAL RH'!C4</f>
         <v/>
       </c>
-      <c r="D11" s="43">
+      <c r="D11" s="48">
         <f>'TOTAL RH'!D4</f>
         <v/>
       </c>
       <c r="E11" s="1" t="n"/>
       <c r="F11" s="1" t="n"/>
       <c r="G11" s="1" t="n"/>
-      <c r="H11" s="42">
+      <c r="H11" s="47">
         <f>'TOTAL RH'!H4</f>
         <v/>
       </c>
-      <c r="I11" s="43">
+      <c r="I11" s="48">
         <f>'TOTAL RH'!I4</f>
         <v/>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="48">
         <f>'TOTAL RH'!J4</f>
         <v/>
       </c>
@@ -6204,30 +6379,30 @@
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="44">
+      <c r="B12" s="49">
         <f>'TOTAL RH'!B5</f>
         <v/>
       </c>
-      <c r="C12" s="45">
+      <c r="C12" s="50">
         <f>'TOTAL RH'!C5</f>
         <v/>
       </c>
-      <c r="D12" s="45">
+      <c r="D12" s="50">
         <f>'TOTAL RH'!D5</f>
         <v/>
       </c>
       <c r="E12" s="1" t="n"/>
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
-      <c r="H12" s="44">
+      <c r="H12" s="49">
         <f>'TOTAL RH'!H5</f>
         <v/>
       </c>
-      <c r="I12" s="45">
+      <c r="I12" s="50">
         <f>'TOTAL RH'!I5</f>
         <v/>
       </c>
-      <c r="J12" s="45">
+      <c r="J12" s="50">
         <f>'TOTAL RH'!J5</f>
         <v/>
       </c>
@@ -6240,30 +6415,30 @@
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="44">
+      <c r="B13" s="49">
         <f>'TOTAL RH'!B6</f>
         <v/>
       </c>
-      <c r="C13" s="45">
+      <c r="C13" s="50">
         <f>'TOTAL RH'!C6</f>
         <v/>
       </c>
-      <c r="D13" s="45">
+      <c r="D13" s="50">
         <f>'TOTAL RH'!D6</f>
         <v/>
       </c>
       <c r="E13" s="1" t="n"/>
       <c r="F13" s="1" t="n"/>
       <c r="G13" s="1" t="n"/>
-      <c r="H13" s="44">
+      <c r="H13" s="49">
         <f>'TOTAL RH'!H6</f>
         <v/>
       </c>
-      <c r="I13" s="45">
+      <c r="I13" s="50">
         <f>'TOTAL RH'!I6</f>
         <v/>
       </c>
-      <c r="J13" s="45">
+      <c r="J13" s="50">
         <f>'TOTAL RH'!J6</f>
         <v/>
       </c>
@@ -6276,30 +6451,30 @@
     </row>
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="44">
+      <c r="B14" s="49">
         <f>'TOTAL RH'!B7</f>
         <v/>
       </c>
-      <c r="C14" s="45">
+      <c r="C14" s="50">
         <f>'TOTAL RH'!C7</f>
         <v/>
       </c>
-      <c r="D14" s="45">
+      <c r="D14" s="50">
         <f>'TOTAL RH'!D7</f>
         <v/>
       </c>
       <c r="E14" s="1" t="n"/>
       <c r="F14" s="1" t="n"/>
       <c r="G14" s="1" t="n"/>
-      <c r="H14" s="44">
+      <c r="H14" s="49">
         <f>'TOTAL RH'!H7</f>
         <v/>
       </c>
-      <c r="I14" s="45">
+      <c r="I14" s="50">
         <f>'TOTAL RH'!I7</f>
         <v/>
       </c>
-      <c r="J14" s="45">
+      <c r="J14" s="50">
         <f>'TOTAL RH'!J7</f>
         <v/>
       </c>
@@ -6312,30 +6487,30 @@
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="46">
+      <c r="B15" s="51">
         <f>'TOTAL RH'!B8</f>
         <v/>
       </c>
-      <c r="C15" s="47">
+      <c r="C15" s="52">
         <f>'TOTAL RH'!C8</f>
         <v/>
       </c>
-      <c r="D15" s="58">
+      <c r="D15" s="65">
         <f>'TOTAL RH'!D8</f>
         <v/>
       </c>
       <c r="E15" s="1" t="n"/>
       <c r="F15" s="1" t="n"/>
       <c r="G15" s="1" t="n"/>
-      <c r="H15" s="46">
+      <c r="H15" s="51">
         <f>'TOTAL RH'!H8</f>
         <v/>
       </c>
-      <c r="I15" s="47">
+      <c r="I15" s="52">
         <f>'TOTAL RH'!I8</f>
         <v/>
       </c>
-      <c r="J15" s="47">
+      <c r="J15" s="52">
         <f>'TOTAL RH'!J8</f>
         <v/>
       </c>
@@ -6348,30 +6523,30 @@
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="44">
+      <c r="B16" s="49">
         <f>'TOTAL RH'!B9</f>
         <v/>
       </c>
-      <c r="C16" s="45">
+      <c r="C16" s="50">
         <f>'TOTAL RH'!C9</f>
         <v/>
       </c>
-      <c r="D16" s="45">
+      <c r="D16" s="50">
         <f>'TOTAL RH'!D9</f>
         <v/>
       </c>
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="1" t="n"/>
       <c r="G16" s="1" t="n"/>
-      <c r="H16" s="44">
+      <c r="H16" s="49">
         <f>'TOTAL RH'!H9</f>
         <v/>
       </c>
-      <c r="I16" s="45">
+      <c r="I16" s="50">
         <f>'TOTAL RH'!I9</f>
         <v/>
       </c>
-      <c r="J16" s="45">
+      <c r="J16" s="50">
         <f>'TOTAL RH'!J9</f>
         <v/>
       </c>
@@ -6384,30 +6559,30 @@
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="46">
+      <c r="B17" s="51">
         <f>'TOTAL RH'!B10</f>
         <v/>
       </c>
-      <c r="C17" s="47">
+      <c r="C17" s="52">
         <f>'TOTAL RH'!C10</f>
         <v/>
       </c>
-      <c r="D17" s="58">
+      <c r="D17" s="65">
         <f>'TOTAL RH'!D10</f>
         <v/>
       </c>
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="n"/>
       <c r="G17" s="1" t="n"/>
-      <c r="H17" s="46">
+      <c r="H17" s="51">
         <f>'TOTAL RH'!H10</f>
         <v/>
       </c>
-      <c r="I17" s="47">
+      <c r="I17" s="52">
         <f>'TOTAL RH'!I10</f>
         <v/>
       </c>
-      <c r="J17" s="47">
+      <c r="J17" s="52">
         <f>'TOTAL RH'!J10</f>
         <v/>
       </c>
@@ -6420,30 +6595,30 @@
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="44">
+      <c r="B18" s="49">
         <f>'TOTAL RH'!B11</f>
         <v/>
       </c>
-      <c r="C18" s="45">
+      <c r="C18" s="50">
         <f>'TOTAL RH'!C11</f>
         <v/>
       </c>
-      <c r="D18" s="45">
+      <c r="D18" s="50">
         <f>'TOTAL RH'!D11</f>
         <v/>
       </c>
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="1" t="n"/>
       <c r="G18" s="1" t="n"/>
-      <c r="H18" s="44">
+      <c r="H18" s="49">
         <f>'TOTAL RH'!H11</f>
         <v/>
       </c>
-      <c r="I18" s="45">
+      <c r="I18" s="50">
         <f>'TOTAL RH'!I11</f>
         <v/>
       </c>
-      <c r="J18" s="45">
+      <c r="J18" s="50">
         <f>'TOTAL RH'!J11</f>
         <v/>
       </c>
@@ -6456,30 +6631,30 @@
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="1" t="n"/>
-      <c r="B19" s="46">
+      <c r="B19" s="51">
         <f>'TOTAL RH'!B12</f>
         <v/>
       </c>
-      <c r="C19" s="47">
+      <c r="C19" s="52">
         <f>'TOTAL RH'!C12</f>
         <v/>
       </c>
-      <c r="D19" s="58">
+      <c r="D19" s="65">
         <f>'TOTAL RH'!D12</f>
         <v/>
       </c>
       <c r="E19" s="1" t="n"/>
       <c r="F19" s="1" t="n"/>
       <c r="G19" s="1" t="n"/>
-      <c r="H19" s="46">
+      <c r="H19" s="51">
         <f>'TOTAL RH'!H12</f>
         <v/>
       </c>
-      <c r="I19" s="47">
+      <c r="I19" s="52">
         <f>'TOTAL RH'!I12</f>
         <v/>
       </c>
-      <c r="J19" s="58">
+      <c r="J19" s="65">
         <f>'TOTAL RH'!J12</f>
         <v/>
       </c>
@@ -6528,7 +6703,7 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="38" t="inlineStr">
+      <c r="B22" s="43" t="inlineStr">
         <is>
           <t>REMARKS  (AV = move code IED/IEP/IER, DMG = move code OER)</t>
         </is>
@@ -6550,21 +6725,21 @@
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="39">
+      <c r="B23" s="44">
         <f>'TOTAL RH'!B2</f>
         <v/>
       </c>
-      <c r="C23" s="56" t="n"/>
-      <c r="D23" s="57" t="n"/>
+      <c r="C23" s="63" t="n"/>
+      <c r="D23" s="64" t="n"/>
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
-      <c r="H23" s="40">
+      <c r="H23" s="45">
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="I23" s="56" t="n"/>
-      <c r="J23" s="57" t="n"/>
+      <c r="I23" s="63" t="n"/>
+      <c r="J23" s="64" t="n"/>
       <c r="K23" s="1" t="n"/>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n"/>
@@ -6574,13 +6749,13 @@
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="34" t="n"/>
-      <c r="C24" s="41" t="inlineStr">
+      <c r="B24" s="33" t="n"/>
+      <c r="C24" s="46" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="D24" s="41" t="inlineStr">
+      <c r="D24" s="46" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
@@ -6588,13 +6763,13 @@
       <c r="E24" s="1" t="n"/>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
-      <c r="H24" s="34" t="n"/>
-      <c r="I24" s="41" t="inlineStr">
+      <c r="H24" s="33" t="n"/>
+      <c r="I24" s="46" t="inlineStr">
         <is>
           <t>20'RE</t>
         </is>
       </c>
-      <c r="J24" s="41" t="inlineStr">
+      <c r="J24" s="46" t="inlineStr">
         <is>
           <t>40'RH</t>
         </is>
@@ -6608,32 +6783,32 @@
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="34" t="inlineStr">
+      <c r="B25" s="33" t="inlineStr">
         <is>
           <t>AV</t>
         </is>
       </c>
-      <c r="C25" s="45">
+      <c r="C25" s="50">
         <f>'TOTAL RH'!C16</f>
         <v/>
       </c>
-      <c r="D25" s="45">
+      <c r="D25" s="50">
         <f>'TOTAL RH'!D16</f>
         <v/>
       </c>
       <c r="E25" s="1" t="n"/>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
-      <c r="H25" s="34" t="inlineStr">
+      <c r="H25" s="33" t="inlineStr">
         <is>
           <t>AV</t>
         </is>
       </c>
-      <c r="I25" s="45">
+      <c r="I25" s="50">
         <f>'TOTAL RH'!I16</f>
         <v/>
       </c>
-      <c r="J25" s="45">
+      <c r="J25" s="50">
         <f>'TOTAL RH'!J16</f>
         <v/>
       </c>
@@ -6646,32 +6821,32 @@
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="34" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>DMG</t>
         </is>
       </c>
-      <c r="C26" s="45">
+      <c r="C26" s="50">
         <f>'TOTAL RH'!C17</f>
         <v/>
       </c>
-      <c r="D26" s="45">
+      <c r="D26" s="50">
         <f>'TOTAL RH'!D17</f>
         <v/>
       </c>
       <c r="E26" s="1" t="n"/>
       <c r="F26" s="1" t="n"/>
       <c r="G26" s="1" t="n"/>
-      <c r="H26" s="34" t="inlineStr">
+      <c r="H26" s="33" t="inlineStr">
         <is>
           <t>DMG</t>
         </is>
       </c>
-      <c r="I26" s="45">
+      <c r="I26" s="50">
         <f>'TOTAL RH'!I17</f>
         <v/>
       </c>
-      <c r="J26" s="45">
+      <c r="J26" s="50">
         <f>'TOTAL RH'!J17</f>
         <v/>
       </c>
@@ -6720,7 +6895,7 @@
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="1" t="n"/>
-      <c r="B29" s="38" t="inlineStr">
+      <c r="B29" s="43" t="inlineStr">
         <is>
           <t>RF SEASONAL — build year</t>
         </is>
@@ -6742,29 +6917,29 @@
     </row>
     <row r="30" ht="13" customHeight="1">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B30" s="39" t="inlineStr">
         <is>
           <t>BKK27 2020-26 BUILT</t>
         </is>
       </c>
-      <c r="C30" s="34" t="n"/>
-      <c r="D30" s="34" t="n"/>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="33" t="n"/>
       <c r="E30" s="1" t="n"/>
-      <c r="F30" s="33" t="inlineStr">
+      <c r="F30" s="39" t="inlineStr">
         <is>
           <t>LCH27 2020-26 BUILT</t>
         </is>
       </c>
-      <c r="G30" s="34" t="n"/>
-      <c r="H30" s="34" t="n"/>
+      <c r="G30" s="33" t="n"/>
+      <c r="H30" s="33" t="n"/>
       <c r="I30" s="1" t="n"/>
-      <c r="J30" s="33" t="inlineStr">
+      <c r="J30" s="39" t="inlineStr">
         <is>
           <t>PEAK BUILD YEAR</t>
         </is>
       </c>
-      <c r="K30" s="34" t="n"/>
-      <c r="L30" s="34" t="n"/>
+      <c r="K30" s="33" t="n"/>
+      <c r="L30" s="33" t="n"/>
       <c r="M30" s="1" t="n"/>
       <c r="N30" s="1" t="n"/>
       <c r="O30" s="1" t="n"/>
@@ -6772,26 +6947,26 @@
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="48">
+      <c r="B31" s="53">
         <f>SUM('TOTAL RH'!D36:D42)+SUM('TOTAL RH'!F36:F42)+SUM('TOTAL RH'!H36:H42)</f>
         <v/>
       </c>
-      <c r="C31" s="34" t="n"/>
-      <c r="D31" s="34" t="n"/>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="33" t="n"/>
       <c r="E31" s="1" t="n"/>
-      <c r="F31" s="49">
+      <c r="F31" s="54">
         <f>SUM('TOTAL RH'!L36:L42)+SUM('TOTAL RH'!N36:N42)+SUM('TOTAL RH'!P36:P42)</f>
         <v/>
       </c>
-      <c r="G31" s="34" t="n"/>
-      <c r="H31" s="34" t="n"/>
+      <c r="G31" s="33" t="n"/>
+      <c r="H31" s="33" t="n"/>
       <c r="I31" s="1" t="n"/>
-      <c r="J31" s="36">
+      <c r="J31" s="41">
         <f>"2021"</f>
         <v/>
       </c>
-      <c r="K31" s="34" t="n"/>
-      <c r="L31" s="34" t="n"/>
+      <c r="K31" s="33" t="n"/>
+      <c r="L31" s="33" t="n"/>
       <c r="M31" s="1" t="n"/>
       <c r="N31" s="1" t="n"/>
       <c r="O31" s="1" t="n"/>
@@ -6799,29 +6974,29 @@
     </row>
     <row r="32" ht="13" customHeight="1">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="37" t="inlineStr">
+      <c r="B32" s="42" t="inlineStr">
         <is>
           <t>of 40'RH on hand</t>
         </is>
       </c>
-      <c r="C32" s="34" t="n"/>
-      <c r="D32" s="34" t="n"/>
+      <c r="C32" s="33" t="n"/>
+      <c r="D32" s="33" t="n"/>
       <c r="E32" s="1" t="n"/>
-      <c r="F32" s="37" t="inlineStr">
+      <c r="F32" s="42" t="inlineStr">
         <is>
           <t>of 40'RH on hand</t>
         </is>
       </c>
-      <c r="G32" s="34" t="n"/>
-      <c r="H32" s="34" t="n"/>
+      <c r="G32" s="33" t="n"/>
+      <c r="H32" s="33" t="n"/>
       <c r="I32" s="1" t="n"/>
-      <c r="J32" s="37" t="inlineStr">
+      <c r="J32" s="42" t="inlineStr">
         <is>
           <t>12 units across both depots</t>
         </is>
       </c>
-      <c r="K32" s="34" t="n"/>
-      <c r="L32" s="34" t="n"/>
+      <c r="K32" s="33" t="n"/>
+      <c r="L32" s="33" t="n"/>
       <c r="M32" s="1" t="n"/>
       <c r="N32" s="1" t="n"/>
       <c r="O32" s="1" t="n"/>
@@ -6849,21 +7024,21 @@
       <c r="A34" s="1" t="n"/>
       <c r="B34" s="39" t="inlineStr">
         <is>
-          <t>BKK27 current mix</t>
-        </is>
-      </c>
-      <c r="C34" s="56" t="n"/>
-      <c r="D34" s="57" t="n"/>
+          <t>DURIAN CARGO  (2021-2026)</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="n"/>
+      <c r="D34" s="33" t="n"/>
       <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="n"/>
-      <c r="G34" s="1" t="n"/>
-      <c r="H34" s="40" t="inlineStr">
-        <is>
-          <t>LCH27 current mix</t>
-        </is>
-      </c>
-      <c r="I34" s="56" t="n"/>
-      <c r="J34" s="57" t="n"/>
+      <c r="F34" s="39" t="inlineStr">
+        <is>
+          <t>NON DURIAN CARGO  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="G34" s="33" t="n"/>
+      <c r="H34" s="33" t="n"/>
+      <c r="I34" s="1" t="n"/>
+      <c r="J34" s="1" t="n"/>
       <c r="K34" s="1" t="n"/>
       <c r="L34" s="1" t="n"/>
       <c r="M34" s="1" t="n"/>
@@ -6873,31 +7048,21 @@
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="34" t="n"/>
-      <c r="C35" s="41" t="inlineStr">
-        <is>
-          <t>22RE</t>
-        </is>
-      </c>
-      <c r="D35" s="41" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
+      <c r="B35" s="55">
+        <f>'TOTAL RH'!B58</f>
+        <v/>
+      </c>
+      <c r="C35" s="33" t="n"/>
+      <c r="D35" s="33" t="n"/>
       <c r="E35" s="1" t="n"/>
-      <c r="F35" s="1" t="n"/>
-      <c r="G35" s="1" t="n"/>
-      <c r="H35" s="34" t="n"/>
-      <c r="I35" s="41" t="inlineStr">
-        <is>
-          <t>22RE</t>
-        </is>
-      </c>
-      <c r="J35" s="41" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
+      <c r="F35" s="56">
+        <f>'TOTAL RH'!G58</f>
+        <v/>
+      </c>
+      <c r="G35" s="33" t="n"/>
+      <c r="H35" s="33" t="n"/>
+      <c r="I35" s="1" t="n"/>
+      <c r="J35" s="1" t="n"/>
       <c r="K35" s="1" t="n"/>
       <c r="L35" s="1" t="n"/>
       <c r="M35" s="1" t="n"/>
@@ -6907,35 +7072,23 @@
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="34" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="C36" s="45">
-        <f>'TOTAL RH'!C53</f>
-        <v/>
-      </c>
-      <c r="D36" s="45">
-        <f>'TOTAL RH'!D53</f>
-        <v/>
-      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>40'RH, both depots combined</t>
+        </is>
+      </c>
+      <c r="C36" s="33" t="n"/>
+      <c r="D36" s="33" t="n"/>
       <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="n"/>
-      <c r="G36" s="1" t="n"/>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="I36" s="45">
-        <f>'TOTAL RH'!K53</f>
-        <v/>
-      </c>
-      <c r="J36" s="45">
-        <f>'TOTAL RH'!L53</f>
-        <v/>
-      </c>
+      <c r="F36" s="42" t="inlineStr">
+        <is>
+          <t>40'RH, both depots combined</t>
+        </is>
+      </c>
+      <c r="G36" s="33" t="n"/>
+      <c r="H36" s="33" t="n"/>
+      <c r="I36" s="1" t="n"/>
+      <c r="J36" s="1" t="n"/>
       <c r="K36" s="1" t="n"/>
       <c r="L36" s="1" t="n"/>
       <c r="M36" s="1" t="n"/>
@@ -6945,35 +7098,15 @@
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="34" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="C37" s="45">
-        <f>'TOTAL RH'!E53</f>
-        <v/>
-      </c>
-      <c r="D37" s="45">
-        <f>'TOTAL RH'!F53</f>
-        <v/>
-      </c>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="n"/>
       <c r="E37" s="1" t="n"/>
       <c r="F37" s="1" t="n"/>
       <c r="G37" s="1" t="n"/>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="I37" s="45">
-        <f>'TOTAL RH'!M53</f>
-        <v/>
-      </c>
-      <c r="J37" s="45">
-        <f>'TOTAL RH'!N53</f>
-        <v/>
-      </c>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="1" t="n"/>
+      <c r="J37" s="1" t="n"/>
       <c r="K37" s="1" t="n"/>
       <c r="L37" s="1" t="n"/>
       <c r="M37" s="1" t="n"/>
@@ -6983,35 +7116,23 @@
     </row>
     <row r="38" ht="13" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="34" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
-      </c>
-      <c r="C38" s="45">
-        <f>'TOTAL RH'!G53</f>
-        <v/>
-      </c>
-      <c r="D38" s="45">
-        <f>'TOTAL RH'!H53</f>
-        <v/>
-      </c>
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>BKK27 current mix</t>
+        </is>
+      </c>
+      <c r="C38" s="63" t="n"/>
+      <c r="D38" s="64" t="n"/>
       <c r="E38" s="1" t="n"/>
       <c r="F38" s="1" t="n"/>
       <c r="G38" s="1" t="n"/>
-      <c r="H38" s="34" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
-      </c>
-      <c r="I38" s="45">
-        <f>'TOTAL RH'!O53</f>
-        <v/>
-      </c>
-      <c r="J38" s="45">
-        <f>'TOTAL RH'!P53</f>
-        <v/>
-      </c>
+      <c r="H38" s="45" t="inlineStr">
+        <is>
+          <t>LCH27 current mix</t>
+        </is>
+      </c>
+      <c r="I38" s="63" t="n"/>
+      <c r="J38" s="64" t="n"/>
       <c r="K38" s="1" t="n"/>
       <c r="L38" s="1" t="n"/>
       <c r="M38" s="1" t="n"/>
@@ -7021,15 +7142,31 @@
     </row>
     <row r="39" ht="13" customHeight="1">
       <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
+      <c r="B39" s="33" t="n"/>
+      <c r="C39" s="46" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
+      <c r="D39" s="46" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
       <c r="E39" s="1" t="n"/>
       <c r="F39" s="1" t="n"/>
       <c r="G39" s="1" t="n"/>
-      <c r="H39" s="1" t="n"/>
-      <c r="I39" s="1" t="n"/>
-      <c r="J39" s="1" t="n"/>
+      <c r="H39" s="33" t="n"/>
+      <c r="I39" s="46" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
+      <c r="J39" s="46" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
       <c r="K39" s="1" t="n"/>
       <c r="L39" s="1" t="n"/>
       <c r="M39" s="1" t="n"/>
@@ -7039,19 +7176,35 @@
     </row>
     <row r="40" ht="13" customHeight="1">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="50" t="inlineStr">
-        <is>
-          <t>Full 2010-2026 Year x Brand x Size breakdown is on the TOTAL RH sheet.</t>
-        </is>
-      </c>
-      <c r="C40" s="1" t="n"/>
-      <c r="D40" s="1" t="n"/>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="C40" s="50">
+        <f>'TOTAL RH'!C53</f>
+        <v/>
+      </c>
+      <c r="D40" s="50">
+        <f>'TOTAL RH'!D53</f>
+        <v/>
+      </c>
       <c r="E40" s="1" t="n"/>
       <c r="F40" s="1" t="n"/>
       <c r="G40" s="1" t="n"/>
-      <c r="H40" s="1" t="n"/>
-      <c r="I40" s="1" t="n"/>
-      <c r="J40" s="1" t="n"/>
+      <c r="H40" s="33" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="I40" s="50">
+        <f>'TOTAL RH'!K53</f>
+        <v/>
+      </c>
+      <c r="J40" s="50">
+        <f>'TOTAL RH'!L53</f>
+        <v/>
+      </c>
       <c r="K40" s="1" t="n"/>
       <c r="L40" s="1" t="n"/>
       <c r="M40" s="1" t="n"/>
@@ -7059,15 +7212,131 @@
       <c r="O40" s="1" t="n"/>
       <c r="P40" s="1" t="n"/>
     </row>
+    <row r="41" ht="13" customHeight="1">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="33" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="C41" s="50">
+        <f>'TOTAL RH'!E53</f>
+        <v/>
+      </c>
+      <c r="D41" s="50">
+        <f>'TOTAL RH'!F53</f>
+        <v/>
+      </c>
+      <c r="E41" s="1" t="n"/>
+      <c r="F41" s="1" t="n"/>
+      <c r="G41" s="1" t="n"/>
+      <c r="H41" s="33" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="I41" s="50">
+        <f>'TOTAL RH'!M53</f>
+        <v/>
+      </c>
+      <c r="J41" s="50">
+        <f>'TOTAL RH'!N53</f>
+        <v/>
+      </c>
+      <c r="K41" s="1" t="n"/>
+      <c r="L41" s="1" t="n"/>
+      <c r="M41" s="1" t="n"/>
+      <c r="N41" s="1" t="n"/>
+      <c r="O41" s="1" t="n"/>
+      <c r="P41" s="1" t="n"/>
+    </row>
+    <row r="42" ht="13" customHeight="1">
+      <c r="A42" s="1" t="n"/>
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="C42" s="50">
+        <f>'TOTAL RH'!G53</f>
+        <v/>
+      </c>
+      <c r="D42" s="50">
+        <f>'TOTAL RH'!H53</f>
+        <v/>
+      </c>
+      <c r="E42" s="1" t="n"/>
+      <c r="F42" s="1" t="n"/>
+      <c r="G42" s="1" t="n"/>
+      <c r="H42" s="33" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="I42" s="50">
+        <f>'TOTAL RH'!O53</f>
+        <v/>
+      </c>
+      <c r="J42" s="50">
+        <f>'TOTAL RH'!P53</f>
+        <v/>
+      </c>
+      <c r="K42" s="1" t="n"/>
+      <c r="L42" s="1" t="n"/>
+      <c r="M42" s="1" t="n"/>
+      <c r="N42" s="1" t="n"/>
+      <c r="O42" s="1" t="n"/>
+      <c r="P42" s="1" t="n"/>
+    </row>
+    <row r="43" ht="13" customHeight="1">
+      <c r="A43" s="1" t="n"/>
+      <c r="B43" s="1" t="n"/>
+      <c r="C43" s="1" t="n"/>
+      <c r="D43" s="1" t="n"/>
+      <c r="E43" s="1" t="n"/>
+      <c r="F43" s="1" t="n"/>
+      <c r="G43" s="1" t="n"/>
+      <c r="H43" s="1" t="n"/>
+      <c r="I43" s="1" t="n"/>
+      <c r="J43" s="1" t="n"/>
+      <c r="K43" s="1" t="n"/>
+      <c r="L43" s="1" t="n"/>
+      <c r="M43" s="1" t="n"/>
+      <c r="N43" s="1" t="n"/>
+      <c r="O43" s="1" t="n"/>
+      <c r="P43" s="1" t="n"/>
+    </row>
+    <row r="44" ht="13" customHeight="1">
+      <c r="A44" s="1" t="n"/>
+      <c r="B44" s="57" t="inlineStr">
+        <is>
+          <t>Full 2010-2026 Year x Brand x Size breakdown is on the TOTAL RH sheet.</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="1" t="n"/>
+      <c r="E44" s="1" t="n"/>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="n"/>
+      <c r="H44" s="1" t="n"/>
+      <c r="I44" s="1" t="n"/>
+      <c r="J44" s="1" t="n"/>
+      <c r="K44" s="1" t="n"/>
+      <c r="L44" s="1" t="n"/>
+      <c r="M44" s="1" t="n"/>
+      <c r="N44" s="1" t="n"/>
+      <c r="O44" s="1" t="n"/>
+      <c r="P44" s="1" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="H38:J38"/>
     <mergeCell ref="B1:P2"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="H34:J34"/>
     <mergeCell ref="H9:J9"/>
-    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B38:D38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Split CARGO classification by depot (BKK27/LCH27)
Both the TOTAL RH section and its linked Dashboard cards now show
4 cards (BKK27/LCH27 x Durian/Non durian) instead of 2 combined
ones, matching the report's per-depot convention elsewhere.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_9-22.xlsx
+++ b/Stock_Daily_Reefer_9-22.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,7 +54,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E7D32"/>
+      <color rgb="002A78D6"/>
       <sz val="20"/>
     </font>
     <font>
@@ -63,7 +63,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="008B979C"/>
+      <color rgb="00EB6834"/>
       <sz val="20"/>
     </font>
     <font>
@@ -105,16 +105,6 @@
       <b val="1"/>
       <color rgb="00EB6834"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="002A78D6"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00EB6834"/>
-      <sz val="20"/>
     </font>
     <font>
       <b val="1"/>
@@ -166,13 +156,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002E7D32"/>
+      <color rgb="002A78D6"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="008B979C"/>
+      <color rgb="00EB6834"/>
       <sz val="11"/>
     </font>
     <font>
@@ -196,18 +186,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000D3B12"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002A78D6"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00EB6834"/>
       <sz val="11"/>
     </font>
     <font>
@@ -434,153 +412,147 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4129,16 +4101,16 @@
         <f>"Stock vs Booking Report - Reefer (20'RE / 40'RH)  as of "&amp;DAY(Control!$B$1)&amp;" "&amp;CHOOSE(MONTH(Control!$B$1),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;" "&amp;YEAR(Control!$B$1)</f>
         <v/>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
-      <c r="F1" s="58" t="n"/>
-      <c r="G1" s="58" t="n"/>
-      <c r="H1" s="58" t="n"/>
-      <c r="I1" s="58" t="n"/>
-      <c r="J1" s="58" t="n"/>
-      <c r="K1" s="59" t="n"/>
+      <c r="B1" s="56" t="n"/>
+      <c r="C1" s="56" t="n"/>
+      <c r="D1" s="56" t="n"/>
+      <c r="E1" s="56" t="n"/>
+      <c r="F1" s="56" t="n"/>
+      <c r="G1" s="56" t="n"/>
+      <c r="H1" s="56" t="n"/>
+      <c r="I1" s="56" t="n"/>
+      <c r="J1" s="56" t="n"/>
+      <c r="K1" s="57" t="n"/>
       <c r="L1" s="1" t="n"/>
       <c r="M1" s="1" t="n"/>
       <c r="N1" s="1" t="n"/>
@@ -4152,8 +4124,8 @@
           <t>BKK27 / BC2</t>
         </is>
       </c>
-      <c r="C2" s="58" t="n"/>
-      <c r="D2" s="59" t="n"/>
+      <c r="C2" s="56" t="n"/>
+      <c r="D2" s="57" t="n"/>
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
@@ -4162,8 +4134,8 @@
           <t>LCH27 / HAST</t>
         </is>
       </c>
-      <c r="I2" s="58" t="n"/>
-      <c r="J2" s="59" t="n"/>
+      <c r="I2" s="56" t="n"/>
+      <c r="J2" s="57" t="n"/>
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
       <c r="M2" s="5" t="inlineStr">
@@ -4435,11 +4407,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C8" s="60">
+      <c r="C8" s="58">
         <f>C4-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="61">
+      <c r="D8" s="59">
         <f>D4-D5-D6-D7</f>
         <v/>
       </c>
@@ -4450,11 +4422,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I8" s="60">
+      <c r="I8" s="58">
         <f>I4-I5-I6-I7</f>
         <v/>
       </c>
-      <c r="J8" s="60">
+      <c r="J8" s="58">
         <f>J4-J5-J6-J7</f>
         <v/>
       </c>
@@ -4533,11 +4505,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C10" s="60">
+      <c r="C10" s="58">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="61">
+      <c r="D10" s="59">
         <f>D8-D9</f>
         <v/>
       </c>
@@ -4548,11 +4520,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I10" s="60">
+      <c r="I10" s="58">
         <f>I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="60">
+      <c r="J10" s="58">
         <f>J8-J9</f>
         <v/>
       </c>
@@ -4621,11 +4593,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C12" s="60">
+      <c r="C12" s="58">
         <f>C10-C11</f>
         <v/>
       </c>
-      <c r="D12" s="61">
+      <c r="D12" s="59">
         <f>D10-D11</f>
         <v/>
       </c>
@@ -4636,11 +4608,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I12" s="60">
+      <c r="I12" s="58">
         <f>I10-I11</f>
         <v/>
       </c>
-      <c r="J12" s="61">
+      <c r="J12" s="59">
         <f>J10-J11</f>
         <v/>
       </c>
@@ -4890,9 +4862,9 @@
           <t>BKK / BC2 (BKK27)</t>
         </is>
       </c>
-      <c r="C20" s="58" t="n"/>
-      <c r="D20" s="58" t="n"/>
-      <c r="E20" s="59" t="n"/>
+      <c r="C20" s="56" t="n"/>
+      <c r="D20" s="56" t="n"/>
+      <c r="E20" s="57" t="n"/>
       <c r="F20" s="1" t="n"/>
       <c r="G20" s="1" t="n"/>
       <c r="H20" s="17" t="inlineStr">
@@ -4900,9 +4872,9 @@
           <t>LCH / HAST (LCH27)</t>
         </is>
       </c>
-      <c r="I20" s="58" t="n"/>
-      <c r="J20" s="58" t="n"/>
-      <c r="K20" s="59" t="n"/>
+      <c r="I20" s="56" t="n"/>
+      <c r="J20" s="56" t="n"/>
+      <c r="K20" s="57" t="n"/>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="n"/>
@@ -4963,7 +4935,7 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="62" t="n"/>
+      <c r="B22" s="60" t="n"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -4981,7 +4953,7 @@
       </c>
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
-      <c r="H22" s="62" t="n"/>
+      <c r="H22" s="60" t="n"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
           <t>45RE</t>
@@ -5318,24 +5290,24 @@
           <t>BKK27 / BC2  —  Stock by Built Year x Brand x Size</t>
         </is>
       </c>
-      <c r="C33" s="58" t="n"/>
-      <c r="D33" s="58" t="n"/>
-      <c r="E33" s="58" t="n"/>
-      <c r="F33" s="58" t="n"/>
-      <c r="G33" s="58" t="n"/>
-      <c r="H33" s="59" t="n"/>
+      <c r="C33" s="56" t="n"/>
+      <c r="D33" s="56" t="n"/>
+      <c r="E33" s="56" t="n"/>
+      <c r="F33" s="56" t="n"/>
+      <c r="G33" s="56" t="n"/>
+      <c r="H33" s="57" t="n"/>
       <c r="I33" s="1" t="n"/>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>LCH27 / HAST  —  Stock by Built Year x Brand x Size</t>
         </is>
       </c>
-      <c r="K33" s="58" t="n"/>
-      <c r="L33" s="58" t="n"/>
-      <c r="M33" s="58" t="n"/>
-      <c r="N33" s="58" t="n"/>
-      <c r="O33" s="58" t="n"/>
-      <c r="P33" s="59" t="n"/>
+      <c r="K33" s="56" t="n"/>
+      <c r="L33" s="56" t="n"/>
+      <c r="M33" s="56" t="n"/>
+      <c r="N33" s="56" t="n"/>
+      <c r="O33" s="56" t="n"/>
+      <c r="P33" s="57" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="1" t="n"/>
@@ -5350,19 +5322,19 @@
           <t>CARRIER</t>
         </is>
       </c>
-      <c r="D34" s="59" t="n"/>
+      <c r="D34" s="57" t="n"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
-      <c r="F34" s="59" t="n"/>
+      <c r="F34" s="57" t="n"/>
       <c r="G34" s="4" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
-      <c r="H34" s="59" t="n"/>
+      <c r="H34" s="57" t="n"/>
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="18" t="inlineStr">
         <is>
@@ -5375,23 +5347,23 @@
           <t>CARRIER</t>
         </is>
       </c>
-      <c r="L34" s="59" t="n"/>
+      <c r="L34" s="57" t="n"/>
       <c r="M34" s="4" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
-      <c r="N34" s="59" t="n"/>
+      <c r="N34" s="57" t="n"/>
       <c r="O34" s="4" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
-      <c r="P34" s="59" t="n"/>
+      <c r="P34" s="57" t="n"/>
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="62" t="n"/>
+      <c r="B35" s="60" t="n"/>
       <c r="C35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
@@ -5423,7 +5395,7 @@
         </is>
       </c>
       <c r="I35" s="1" t="n"/>
-      <c r="J35" s="62" t="n"/>
+      <c r="J35" s="60" t="n"/>
       <c r="K35" s="22" t="inlineStr">
         <is>
           <t>20'RE</t>
@@ -5981,7 +5953,7 @@
       <c r="A56" s="1" t="n"/>
       <c r="B56" s="31" t="inlineStr">
         <is>
-          <t>CARGO CLASSIFICATION  (both depots, 40'RH stock, by Built Year)</t>
+          <t>CARGO CLASSIFICATION  (40'RH stock by Built Year, per depot)</t>
         </is>
       </c>
       <c r="C56" s="1" t="n"/>
@@ -6003,77 +5975,99 @@
       <c r="A57" s="1" t="n"/>
       <c r="B57" s="32" t="inlineStr">
         <is>
-          <t>DURIAN  (built 2021-2026)</t>
+          <t>BKK27 DURIAN  (2021-2026)</t>
         </is>
       </c>
       <c r="C57" s="33" t="n"/>
       <c r="D57" s="33" t="n"/>
-      <c r="E57" s="33" t="n"/>
-      <c r="F57" s="1" t="n"/>
-      <c r="G57" s="32" t="inlineStr">
-        <is>
-          <t>NON DURIAN  (built ≤ 2020)</t>
-        </is>
-      </c>
+      <c r="E57" s="1" t="n"/>
+      <c r="F57" s="32" t="inlineStr">
+        <is>
+          <t>BKK27 NON DURIAN  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="G57" s="33" t="n"/>
       <c r="H57" s="33" t="n"/>
-      <c r="I57" s="33" t="n"/>
-      <c r="J57" s="33" t="n"/>
-      <c r="K57" s="1" t="n"/>
-      <c r="L57" s="1" t="n"/>
+      <c r="I57" s="1" t="n"/>
+      <c r="J57" s="32" t="inlineStr">
+        <is>
+          <t>LCH27 DURIAN  (2021-2026)</t>
+        </is>
+      </c>
+      <c r="K57" s="33" t="n"/>
+      <c r="L57" s="33" t="n"/>
       <c r="M57" s="1" t="n"/>
-      <c r="N57" s="1" t="n"/>
-      <c r="O57" s="1" t="n"/>
-      <c r="P57" s="1" t="n"/>
+      <c r="N57" s="32" t="inlineStr">
+        <is>
+          <t>LCH27 NON DURIAN  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="O57" s="33" t="n"/>
+      <c r="P57" s="33" t="n"/>
     </row>
     <row r="58" ht="13" customHeight="1">
       <c r="A58" s="1" t="n"/>
       <c r="B58" s="34">
-        <f>SUM(D36:D41)+SUM(F36:F41)+SUM(H36:H41)+SUM(L36:L41)+SUM(N36:N41)+SUM(P36:P41)</f>
+        <f>SUM(D36:D41)+SUM(F36:F41)+SUM(H36:H41)</f>
         <v/>
       </c>
       <c r="C58" s="33" t="n"/>
       <c r="D58" s="33" t="n"/>
-      <c r="E58" s="33" t="n"/>
-      <c r="F58" s="1" t="n"/>
-      <c r="G58" s="35">
-        <f>SUM(D42:D52)+SUM(F42:F52)+SUM(H42:H52)+SUM(L42:L52)+SUM(N42:N52)+SUM(P42:P52)</f>
-        <v/>
-      </c>
+      <c r="E58" s="1" t="n"/>
+      <c r="F58" s="34">
+        <f>SUM(D42:D52)+SUM(F42:F52)+SUM(H42:H52)</f>
+        <v/>
+      </c>
+      <c r="G58" s="33" t="n"/>
       <c r="H58" s="33" t="n"/>
-      <c r="I58" s="33" t="n"/>
-      <c r="J58" s="33" t="n"/>
-      <c r="K58" s="1" t="n"/>
-      <c r="L58" s="1" t="n"/>
+      <c r="I58" s="1" t="n"/>
+      <c r="J58" s="35">
+        <f>SUM(L36:L41)+SUM(N36:N41)+SUM(P36:P41)</f>
+        <v/>
+      </c>
+      <c r="K58" s="33" t="n"/>
+      <c r="L58" s="33" t="n"/>
       <c r="M58" s="1" t="n"/>
-      <c r="N58" s="1" t="n"/>
-      <c r="O58" s="1" t="n"/>
-      <c r="P58" s="1" t="n"/>
+      <c r="N58" s="35">
+        <f>SUM(L42:L52)+SUM(N42:N52)+SUM(P42:P52)</f>
+        <v/>
+      </c>
+      <c r="O58" s="33" t="n"/>
+      <c r="P58" s="33" t="n"/>
     </row>
     <row r="59" ht="13" customHeight="1">
       <c r="A59" s="1" t="n"/>
       <c r="B59" s="36" t="inlineStr">
         <is>
-          <t>40'RH, both depots combined</t>
+          <t>40'RH stock</t>
         </is>
       </c>
       <c r="C59" s="33" t="n"/>
       <c r="D59" s="33" t="n"/>
-      <c r="E59" s="33" t="n"/>
-      <c r="F59" s="1" t="n"/>
-      <c r="G59" s="36" t="inlineStr">
-        <is>
-          <t>40'RH, both depots combined</t>
-        </is>
-      </c>
+      <c r="E59" s="1" t="n"/>
+      <c r="F59" s="36" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="G59" s="33" t="n"/>
       <c r="H59" s="33" t="n"/>
-      <c r="I59" s="33" t="n"/>
-      <c r="J59" s="33" t="n"/>
-      <c r="K59" s="1" t="n"/>
-      <c r="L59" s="1" t="n"/>
+      <c r="I59" s="1" t="n"/>
+      <c r="J59" s="36" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="K59" s="33" t="n"/>
+      <c r="L59" s="33" t="n"/>
       <c r="M59" s="1" t="n"/>
-      <c r="N59" s="1" t="n"/>
-      <c r="O59" s="1" t="n"/>
-      <c r="P59" s="1" t="n"/>
+      <c r="N59" s="36" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="O59" s="33" t="n"/>
+      <c r="P59" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -6289,8 +6283,8 @@
         <f>'TOTAL RH'!B2</f>
         <v/>
       </c>
-      <c r="C9" s="63" t="n"/>
-      <c r="D9" s="64" t="n"/>
+      <c r="C9" s="61" t="n"/>
+      <c r="D9" s="62" t="n"/>
       <c r="E9" s="1" t="n"/>
       <c r="F9" s="1" t="n"/>
       <c r="G9" s="1" t="n"/>
@@ -6298,8 +6292,8 @@
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="I9" s="63" t="n"/>
-      <c r="J9" s="64" t="n"/>
+      <c r="I9" s="61" t="n"/>
+      <c r="J9" s="62" t="n"/>
       <c r="K9" s="1" t="n"/>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
@@ -6495,7 +6489,7 @@
         <f>'TOTAL RH'!C8</f>
         <v/>
       </c>
-      <c r="D15" s="65">
+      <c r="D15" s="63">
         <f>'TOTAL RH'!D8</f>
         <v/>
       </c>
@@ -6567,7 +6561,7 @@
         <f>'TOTAL RH'!C10</f>
         <v/>
       </c>
-      <c r="D17" s="65">
+      <c r="D17" s="63">
         <f>'TOTAL RH'!D10</f>
         <v/>
       </c>
@@ -6639,7 +6633,7 @@
         <f>'TOTAL RH'!C12</f>
         <v/>
       </c>
-      <c r="D19" s="65">
+      <c r="D19" s="63">
         <f>'TOTAL RH'!D12</f>
         <v/>
       </c>
@@ -6654,7 +6648,7 @@
         <f>'TOTAL RH'!I12</f>
         <v/>
       </c>
-      <c r="J19" s="65">
+      <c r="J19" s="63">
         <f>'TOTAL RH'!J12</f>
         <v/>
       </c>
@@ -6729,8 +6723,8 @@
         <f>'TOTAL RH'!B2</f>
         <v/>
       </c>
-      <c r="C23" s="63" t="n"/>
-      <c r="D23" s="64" t="n"/>
+      <c r="C23" s="61" t="n"/>
+      <c r="D23" s="62" t="n"/>
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
@@ -6738,8 +6732,8 @@
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="I23" s="63" t="n"/>
-      <c r="J23" s="64" t="n"/>
+      <c r="I23" s="61" t="n"/>
+      <c r="J23" s="62" t="n"/>
       <c r="K23" s="1" t="n"/>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n"/>
@@ -7024,7 +7018,7 @@
       <c r="A34" s="1" t="n"/>
       <c r="B34" s="39" t="inlineStr">
         <is>
-          <t>DURIAN CARGO  (2021-2026)</t>
+          <t>BKK27 DURIAN  (2021-2026)</t>
         </is>
       </c>
       <c r="C34" s="33" t="n"/>
@@ -7032,49 +7026,63 @@
       <c r="E34" s="1" t="n"/>
       <c r="F34" s="39" t="inlineStr">
         <is>
-          <t>NON DURIAN CARGO  (≤ 2020)</t>
+          <t>BKK27 NON DURIAN  (≤ 2020)</t>
         </is>
       </c>
       <c r="G34" s="33" t="n"/>
       <c r="H34" s="33" t="n"/>
       <c r="I34" s="1" t="n"/>
-      <c r="J34" s="1" t="n"/>
-      <c r="K34" s="1" t="n"/>
-      <c r="L34" s="1" t="n"/>
+      <c r="J34" s="39" t="inlineStr">
+        <is>
+          <t>LCH27 DURIAN  (2021-2026)</t>
+        </is>
+      </c>
+      <c r="K34" s="33" t="n"/>
+      <c r="L34" s="33" t="n"/>
       <c r="M34" s="1" t="n"/>
-      <c r="N34" s="1" t="n"/>
-      <c r="O34" s="1" t="n"/>
-      <c r="P34" s="1" t="n"/>
+      <c r="N34" s="39" t="inlineStr">
+        <is>
+          <t>LCH27 NON DURIAN  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="O34" s="33" t="n"/>
+      <c r="P34" s="33" t="n"/>
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="55">
+      <c r="B35" s="53">
         <f>'TOTAL RH'!B58</f>
         <v/>
       </c>
       <c r="C35" s="33" t="n"/>
       <c r="D35" s="33" t="n"/>
       <c r="E35" s="1" t="n"/>
-      <c r="F35" s="56">
-        <f>'TOTAL RH'!G58</f>
+      <c r="F35" s="53">
+        <f>'TOTAL RH'!F58</f>
         <v/>
       </c>
       <c r="G35" s="33" t="n"/>
       <c r="H35" s="33" t="n"/>
       <c r="I35" s="1" t="n"/>
-      <c r="J35" s="1" t="n"/>
-      <c r="K35" s="1" t="n"/>
-      <c r="L35" s="1" t="n"/>
+      <c r="J35" s="54">
+        <f>'TOTAL RH'!J58</f>
+        <v/>
+      </c>
+      <c r="K35" s="33" t="n"/>
+      <c r="L35" s="33" t="n"/>
       <c r="M35" s="1" t="n"/>
-      <c r="N35" s="1" t="n"/>
-      <c r="O35" s="1" t="n"/>
-      <c r="P35" s="1" t="n"/>
+      <c r="N35" s="54">
+        <f>'TOTAL RH'!N58</f>
+        <v/>
+      </c>
+      <c r="O35" s="33" t="n"/>
+      <c r="P35" s="33" t="n"/>
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" s="1" t="n"/>
       <c r="B36" s="42" t="inlineStr">
         <is>
-          <t>40'RH, both depots combined</t>
+          <t>40'RH stock</t>
         </is>
       </c>
       <c r="C36" s="33" t="n"/>
@@ -7082,19 +7090,27 @@
       <c r="E36" s="1" t="n"/>
       <c r="F36" s="42" t="inlineStr">
         <is>
-          <t>40'RH, both depots combined</t>
+          <t>40'RH stock</t>
         </is>
       </c>
       <c r="G36" s="33" t="n"/>
       <c r="H36" s="33" t="n"/>
       <c r="I36" s="1" t="n"/>
-      <c r="J36" s="1" t="n"/>
-      <c r="K36" s="1" t="n"/>
-      <c r="L36" s="1" t="n"/>
+      <c r="J36" s="42" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="K36" s="33" t="n"/>
+      <c r="L36" s="33" t="n"/>
       <c r="M36" s="1" t="n"/>
-      <c r="N36" s="1" t="n"/>
-      <c r="O36" s="1" t="n"/>
-      <c r="P36" s="1" t="n"/>
+      <c r="N36" s="42" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="O36" s="33" t="n"/>
+      <c r="P36" s="33" t="n"/>
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="1" t="n"/>
@@ -7121,8 +7137,8 @@
           <t>BKK27 current mix</t>
         </is>
       </c>
-      <c r="C38" s="63" t="n"/>
-      <c r="D38" s="64" t="n"/>
+      <c r="C38" s="61" t="n"/>
+      <c r="D38" s="62" t="n"/>
       <c r="E38" s="1" t="n"/>
       <c r="F38" s="1" t="n"/>
       <c r="G38" s="1" t="n"/>
@@ -7131,8 +7147,8 @@
           <t>LCH27 current mix</t>
         </is>
       </c>
-      <c r="I38" s="63" t="n"/>
-      <c r="J38" s="64" t="n"/>
+      <c r="I38" s="61" t="n"/>
+      <c r="J38" s="62" t="n"/>
       <c r="K38" s="1" t="n"/>
       <c r="L38" s="1" t="n"/>
       <c r="M38" s="1" t="n"/>
@@ -7308,7 +7324,7 @@
     </row>
     <row r="44" ht="13" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="57" t="inlineStr">
+      <c r="B44" s="55" t="inlineStr">
         <is>
           <t>Full 2010-2026 Year x Brand x Size breakdown is on the TOTAL RH sheet.</t>
         </is>

</xml_diff>